<commit_message>
Use 10-digit internal item codes starting with 9
Codes starting with 2 are read as weighing-scale barcodes, which turned part of the code into decimals on import.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/sample/expected-output.xlsx
+++ b/tests/sample/expected-output.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>2000000000015</t>
+          <t>9000000001</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2000000000022</t>
+          <t>9000000002</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2000000000039</t>
+          <t>9000000003</t>
         </is>
       </c>
       <c r="C5" s="2" t="n"/>

</xml_diff>

<commit_message>
Label-reading rules and 10-digit internal item codes (#6)
* Add rules for reading faulty printed labels

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>

* Use 10-digit internal item codes starting with 9

Codes starting with 2 are read as weighing-scale barcodes, which turned part of the code into decimals on import.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>

---------

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/sample/expected-output.xlsx
+++ b/tests/sample/expected-output.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>2000000000015</t>
+          <t>9000000001</t>
         </is>
       </c>
       <c r="C2" s="2" t="n"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2000000000022</t>
+          <t>9000000002</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2000000000039</t>
+          <t>9000000003</t>
         </is>
       </c>
       <c r="C5" s="2" t="n"/>

</xml_diff>

<commit_message>
Remove template sample-row formatting from generated files
Only the header row keeps its borders and colour; the sample rows and note rows are cleared with their formatting.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/sample/expected-output.xlsx
+++ b/tests/sample/expected-output.xlsx
@@ -92,7 +92,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -572,7 +572,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Super Friend Peacock Notebook 112 Pages</t>
         </is>
@@ -582,37 +582,24 @@
           <t>9000000001</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>40</v>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n">
+      <c r="G2" t="n">
         <v>35</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" t="n">
         <v>20</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" t="n">
         <v>30</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" t="n">
         <v>10</v>
       </c>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n">
+      <c r="N2" t="n">
         <v>120</v>
       </c>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
@@ -621,7 +608,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Sahitya Sangam Vaibhava Lakshmi Vratamu</t>
         </is>
@@ -631,37 +618,24 @@
           <t>9789392411144</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>15</v>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n">
+      <c r="G3" t="n">
         <v>10</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" t="n">
         <v>8</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n">
+      <c r="N3" t="n">
         <v>350</v>
       </c>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n"/>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="n"/>
-      <c r="U3" s="2" t="n"/>
       <c r="AE3" t="inlineStr">
         <is>
           <t>Stationery/General</t>
@@ -669,7 +643,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Sri Vinayaka Vratakalpamu</t>
         </is>
@@ -679,37 +653,24 @@
           <t>9000000002</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>25</v>
       </c>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n">
+      <c r="G4" t="n">
         <v>25</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" t="n">
         <v>12.5</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" t="n">
         <v>10</v>
       </c>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n">
+      <c r="N4" t="n">
         <v>50</v>
       </c>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="n"/>
-      <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="n"/>
-      <c r="U4" s="2" t="n"/>
       <c r="AE4" t="inlineStr">
         <is>
           <t>Books</t>
@@ -717,7 +678,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Kapil Duplicating Bill Book No. 04</t>
         </is>
@@ -727,37 +688,24 @@
           <t>9000000003</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>60</v>
       </c>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n">
+      <c r="G5" t="n">
         <v>50</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" t="n">
         <v>40.5</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" t="n">
         <v>45</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n">
+      <c r="N5" t="n">
         <v>60</v>
       </c>
-      <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="n"/>
-      <c r="R5" s="2" t="n"/>
-      <c r="S5" s="2" t="n"/>
-      <c r="T5" s="2" t="n"/>
-      <c r="U5" s="2" t="n"/>
       <c r="AE5" t="inlineStr">
         <is>
           <t>Toys</t>
@@ -765,27 +713,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="n"/>
-      <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="n"/>
-      <c r="U6" s="2" t="n"/>
       <c r="AE6" t="inlineStr">
         <is>
           <t>Decorative Items</t>
@@ -793,27 +720,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="n"/>
-      <c r="U7" s="2" t="n"/>
       <c r="AE7" t="inlineStr">
         <is>
           <t>Prathap plastic pencil box</t>
@@ -821,27 +727,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="n"/>
-      <c r="U8" s="2" t="n"/>
       <c r="AE8" t="inlineStr">
         <is>
           <t>Electronics</t>
@@ -849,27 +734,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="n"/>
       <c r="AE9" t="inlineStr">
         <is>
           <t>Pooja Books/Devotional</t>
@@ -877,27 +741,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3" t="n"/>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3" t="n"/>
-      <c r="U10" s="3" t="n"/>
       <c r="AE10" t="inlineStr">
         <is>
           <t>Account Books</t>

</xml_diff>

<commit_message>
Remove template sample-row formatting from generated files (#7)
Only the header row keeps its borders and colour; the sample rows and note rows are cleared with their formatting.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/sample/expected-output.xlsx
+++ b/tests/sample/expected-output.xlsx
@@ -92,7 +92,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -572,7 +572,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Super Friend Peacock Notebook 112 Pages</t>
         </is>
@@ -582,37 +582,24 @@
           <t>9000000001</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>40</v>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n">
+      <c r="G2" t="n">
         <v>35</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" t="n">
         <v>20</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" t="n">
         <v>30</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" t="n">
         <v>10</v>
       </c>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n">
+      <c r="N2" t="n">
         <v>120</v>
       </c>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
@@ -621,7 +608,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Sahitya Sangam Vaibhava Lakshmi Vratamu</t>
         </is>
@@ -631,37 +618,24 @@
           <t>9789392411144</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>15</v>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n">
+      <c r="G3" t="n">
         <v>10</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" t="n">
         <v>8</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n">
+      <c r="N3" t="n">
         <v>350</v>
       </c>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n"/>
-      <c r="Q3" s="2" t="n"/>
-      <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="n"/>
-      <c r="U3" s="2" t="n"/>
       <c r="AE3" t="inlineStr">
         <is>
           <t>Stationery/General</t>
@@ -669,7 +643,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Sri Vinayaka Vratakalpamu</t>
         </is>
@@ -679,37 +653,24 @@
           <t>9000000002</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>25</v>
       </c>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n">
+      <c r="G4" t="n">
         <v>25</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" t="n">
         <v>12.5</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" t="n">
         <v>10</v>
       </c>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n">
+      <c r="N4" t="n">
         <v>50</v>
       </c>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="n"/>
-      <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="n"/>
-      <c r="U4" s="2" t="n"/>
       <c r="AE4" t="inlineStr">
         <is>
           <t>Books</t>
@@ -717,7 +678,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Kapil Duplicating Bill Book No. 04</t>
         </is>
@@ -727,37 +688,24 @@
           <t>9000000003</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>60</v>
       </c>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n">
+      <c r="G5" t="n">
         <v>50</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" t="n">
         <v>40.5</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" t="n">
         <v>45</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n">
+      <c r="N5" t="n">
         <v>60</v>
       </c>
-      <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="n"/>
-      <c r="R5" s="2" t="n"/>
-      <c r="S5" s="2" t="n"/>
-      <c r="T5" s="2" t="n"/>
-      <c r="U5" s="2" t="n"/>
       <c r="AE5" t="inlineStr">
         <is>
           <t>Toys</t>
@@ -765,27 +713,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="n"/>
-      <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="n"/>
-      <c r="U6" s="2" t="n"/>
       <c r="AE6" t="inlineStr">
         <is>
           <t>Decorative Items</t>
@@ -793,27 +720,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="n"/>
-      <c r="U7" s="2" t="n"/>
       <c r="AE7" t="inlineStr">
         <is>
           <t>Prathap plastic pencil box</t>
@@ -821,27 +727,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="n"/>
-      <c r="U8" s="2" t="n"/>
       <c r="AE8" t="inlineStr">
         <is>
           <t>Electronics</t>
@@ -849,27 +734,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3" t="n"/>
-      <c r="U9" s="3" t="n"/>
       <c r="AE9" t="inlineStr">
         <is>
           <t>Pooja Books/Devotional</t>
@@ -877,27 +741,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3" t="n"/>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3" t="n"/>
-      <c r="U10" s="3" t="n"/>
       <c r="AE10" t="inlineStr">
         <is>
           <t>Account Books</t>

</xml_diff>